<commit_message>
feat: categories sheet — 카테고리 정의를 Google Sheets로 관리
- DEFAULT_CATEGORIES 배열 추가 (key, name, color, filterLabel)
- CC, CN, FILTER_BTNS를 const→let으로 변경, buildCategoryMaps()로 동적 구성
- reloadData()에서 'categories' 시트를 4개 시트와 병렬 fetch
- 시트 데이터 있으면 카테고리 맵 재구성, 없으면 DEFAULT_CATEGORIES 사용
- Excel 템플릿에 categories 시트 추가 (key/name/color/filterLabel, 컬러 셀 배경 표시)
- Settings 힌트에 categories 시트명 추가

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/japan-wbs-template.xlsx
+++ b/japan-wbs-template.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="tasks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="decisions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="resources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="categories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="tasks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="resources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0&quot;주&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +70,15 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -109,6 +117,46 @@
         <bgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3B82F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7C3AED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA78BFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC4B5FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6D28D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF10B981"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF59E0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEF4444"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -122,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -159,6 +207,43 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -237,6 +322,31 @@
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>System</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>타임라인에 표시될 카테고리 전체 이름</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>HEX 색상코드 (#RRGGBB 형식)</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>필터 버튼에 표시될 짧은 이름</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>System</author>
@@ -768,20 +878,26 @@
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - decisions: 주요 의사결정 항목 (8행)</t>
+          <t xml:space="preserve">  - categories: 태스크 카테고리 정의 (색상·필터 레이블)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - decisions: 주요 의사결정 항목 (8행)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="6" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - resources: 팀별 리소스 현황 (7행)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="6" customHeight="1"/>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>■ 주의사항</t>
         </is>
@@ -790,7 +906,7 @@
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - 시트 이름(tasks / decisions / resources)을 변경하지 마세요</t>
+          <t xml:space="preserve">  - 시트 이름(tasks / categories / decisions / resources)을 변경하지 마세요</t>
         </is>
       </c>
     </row>
@@ -836,6 +952,225 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>filterLabel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>A. 기존솔루션 현지화</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>#3B82F6</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>기존솔루션</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B3" s="18" t="inlineStr">
+        <is>
+          <t>B-1순위: 핵심기능·노쇼방지</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>#7C3AED</t>
+        </is>
+      </c>
+      <c r="D3" s="18" t="inlineStr">
+        <is>
+          <t>1순위</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>B-2순위: 운영효율</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>#A78BFA</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>2순위</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>B-3순위: 부가가치</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>#C4B5FD</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>3순위</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>B-기반: 인프라/법적</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>#6D28D9</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>인프라</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>C. 회원관리 체계</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>#10B981</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>회원</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>D. 사업/법무</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>#F59E0B</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>사업</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>QA·런칭</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>#EF4444</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3185,7 +3520,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3449,7 +3784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>